<commit_message>
Updated cure data (v47)
</commit_message>
<xml_diff>
--- a/src/data/routekaart_status_cure.xlsx
+++ b/src/data/routekaart_status_cure.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF744C0A-D195-4964-9221-4ED8670C9A47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFAE8F31-D786-4C1E-9A2A-EEAA5BB36032}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5895" yWindow="2610" windowWidth="31590" windowHeight="17385" xr2:uid="{8CE8C91A-5D2B-429A-9150-16FF2E6CA716}"/>
+    <workbookView xWindow="6840" yWindow="1700" windowWidth="23760" windowHeight="18690" xr2:uid="{8CE8C91A-5D2B-429A-9150-16FF2E6CA716}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -253,10 +253,10 @@
     <t>Radiotherapiegroep</t>
   </si>
   <si>
-    <t>Frisius MC locatie Leeuwarden</t>
-  </si>
-  <si>
-    <t>Frisius MC locatie Heerenveen</t>
+    <t>Frisius MC</t>
+  </si>
+  <si>
+    <t>Medisch Centrum Leeuwarden</t>
   </si>
 </sst>
 </file>
@@ -618,13 +618,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7F40E7E-2647-4F3F-8219-3AF753B4033B}">
   <dimension ref="A1:B73"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="41.7109375" customWidth="1"/>
-    <col min="2" max="2" width="33.28515625" customWidth="1"/>
+    <col min="1" max="1" width="41.7265625" customWidth="1"/>
+    <col min="2" max="2" width="33.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>64</v>
       </c>
@@ -632,7 +632,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>67</v>
       </c>
@@ -640,7 +640,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>40</v>
       </c>
@@ -648,7 +648,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -656,7 +656,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -664,7 +664,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -672,7 +672,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>66</v>
       </c>
@@ -680,7 +680,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -688,7 +688,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>41</v>
       </c>
@@ -696,7 +696,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -704,7 +704,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>27</v>
       </c>
@@ -712,15 +712,15 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>65</v>
       </c>
       <c r="B12" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -728,7 +728,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>58</v>
       </c>
@@ -736,7 +736,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>42</v>
       </c>
@@ -744,7 +744,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>28</v>
       </c>
@@ -752,7 +752,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>43</v>
       </c>
@@ -760,7 +760,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>37</v>
       </c>
@@ -768,7 +768,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -776,359 +776,359 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
+        <v>74</v>
+      </c>
+      <c r="B20" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
         <v>6</v>
       </c>
-      <c r="B20" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+      <c r="B21" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
         <v>29</v>
       </c>
-      <c r="B21" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+      <c r="B22" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
         <v>72</v>
       </c>
-      <c r="B22" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+      <c r="B23" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
         <v>8</v>
       </c>
-      <c r="B23" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+      <c r="B24" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
         <v>44</v>
       </c>
-      <c r="B24" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+      <c r="B25" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
         <v>9</v>
       </c>
-      <c r="B25" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+      <c r="B26" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
         <v>45</v>
       </c>
-      <c r="B26" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+      <c r="B27" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
         <v>69</v>
       </c>
-      <c r="B27" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+      <c r="B28" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
         <v>30</v>
       </c>
-      <c r="B28" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+      <c r="B29" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
         <v>31</v>
       </c>
-      <c r="B29" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+      <c r="B30" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
         <v>1</v>
       </c>
-      <c r="B30" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+      <c r="B31" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
         <v>10</v>
       </c>
-      <c r="B31" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+      <c r="B32" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
         <v>68</v>
       </c>
-      <c r="B32" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>74</v>
-      </c>
       <c r="B33" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
+        <v>75</v>
+      </c>
+      <c r="B34" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
         <v>12</v>
       </c>
-      <c r="B34" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+      <c r="B35" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
         <v>32</v>
       </c>
-      <c r="B35" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+      <c r="B36" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
         <v>38</v>
       </c>
-      <c r="B36" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+      <c r="B37" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
         <v>11</v>
       </c>
-      <c r="B37" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+      <c r="B38" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
         <v>39</v>
       </c>
-      <c r="B38" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+      <c r="B39" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
         <v>15</v>
       </c>
-      <c r="B39" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+      <c r="B40" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
         <v>33</v>
       </c>
-      <c r="B40" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+      <c r="B41" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
         <v>46</v>
       </c>
-      <c r="B41" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
+      <c r="B42" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
         <v>59</v>
       </c>
-      <c r="B42" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
+      <c r="B43" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
         <v>47</v>
       </c>
-      <c r="B43" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
+      <c r="B44" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
         <v>73</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B45" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
         <v>70</v>
       </c>
-      <c r="B45" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
+      <c r="B46" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
         <v>13</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B47" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
         <v>60</v>
       </c>
-      <c r="B47" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
+      <c r="B48" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
         <v>34</v>
       </c>
-      <c r="B48" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
+      <c r="B49" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
         <v>61</v>
       </c>
-      <c r="B49" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
+      <c r="B50" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
         <v>48</v>
       </c>
-      <c r="B50" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
+      <c r="B51" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
         <v>26</v>
       </c>
-      <c r="B51" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
+      <c r="B52" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
         <v>14</v>
       </c>
-      <c r="B52" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
+      <c r="B53" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
         <v>49</v>
       </c>
-      <c r="B53" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
+      <c r="B54" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
         <v>19</v>
       </c>
-      <c r="B54" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
+      <c r="B55" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
         <v>7</v>
       </c>
-      <c r="B55" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
+      <c r="B56" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
         <v>50</v>
       </c>
-      <c r="B56" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
+      <c r="B57" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
         <v>51</v>
       </c>
-      <c r="B57" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
+      <c r="B58" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
         <v>52</v>
       </c>
-      <c r="B58" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
+      <c r="B59" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
         <v>53</v>
       </c>
-      <c r="B59" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
+      <c r="B60" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
         <v>17</v>
       </c>
-      <c r="B60" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
+      <c r="B61" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
         <v>54</v>
       </c>
-      <c r="B61" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
+      <c r="B62" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
         <v>62</v>
       </c>
-      <c r="B62" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>75</v>
-      </c>
       <c r="B63" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>22</v>
       </c>
@@ -1136,7 +1136,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>55</v>
       </c>
@@ -1144,7 +1144,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>56</v>
       </c>
@@ -1152,7 +1152,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>35</v>
       </c>
@@ -1160,7 +1160,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>20</v>
       </c>
@@ -1168,7 +1168,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>21</v>
       </c>
@@ -1176,7 +1176,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>36</v>
       </c>
@@ -1184,7 +1184,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>63</v>
       </c>
@@ -1192,7 +1192,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>71</v>
       </c>
@@ -1200,7 +1200,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>57</v>
       </c>

</xml_diff>

<commit_message>
Updated cure data (v49)
</commit_message>
<xml_diff>
--- a/src/data/routekaart_status_cure.xlsx
+++ b/src/data/routekaart_status_cure.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFAE8F31-D786-4C1E-9A2A-EEAA5BB36032}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{561EBB31-AF43-42C0-82B3-0EBC8A1914EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6840" yWindow="1700" windowWidth="23760" windowHeight="18690" xr2:uid="{8CE8C91A-5D2B-429A-9150-16FF2E6CA716}"/>
+    <workbookView xWindow="3620" yWindow="1520" windowWidth="31120" windowHeight="19700" xr2:uid="{8CE8C91A-5D2B-429A-9150-16FF2E6CA716}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -997,7 +997,7 @@
         <v>13</v>
       </c>
       <c r="B47" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.35">

</xml_diff>